<commit_message>
GD4-GD5: phan tich khoi dau, NFR, elicitation results, product backlog, story map
</commit_message>
<xml_diff>
--- a/00_Admin/HL-OMS_Registers.xlsx
+++ b/00_Admin/HL-OMS_Registers.xlsx
@@ -1721,7 +1721,7 @@
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="31.5" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="38.7" customWidth="1" min="6" max="6"/>
+    <col width="40.5" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Phỏng vấn + Phân tích giao diện</t>
+          <t>Phỏng vấn + Interface analysis (user testing)</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">

</xml_diff>

<commit_message>
GD10: UAT 99 TC + report, RTM tu dong (0 lo hong), BRD, SRS, User Guide, Go-live Plan, Business Case, pitch deck, ban Word; build_all
</commit_message>
<xml_diff>
--- a/00_Admin/HL-OMS_Registers.xlsx
+++ b/00_Admin/HL-OMS_Registers.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assumption Log'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Log'!$A$1:$K$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Decision Log'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Log'!$A$1:$K$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Decision Log'!$A$1:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1713,7 +1713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.5" customWidth="1" min="1" max="1"/>
@@ -1726,7 +1726,7 @@
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="9.9" customWidth="1" min="11" max="11"/>
+    <col width="10.8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4066,8 +4066,65 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>(6) Khác</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Q-041</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Thứ Hai 26/04/2027 (sau Anzac Day) có là ngày lễ NSW để áp phụ thu không?</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu ngày lễ (BR-10)</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>MGR</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Review tài liệu (trang NSW Government)</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Nguồn thứ cấp mâu thuẫn; hạn xác nhận 01/04/2027</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>holidays.csv</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K41"/>
+  <autoFilter ref="A1:K42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4078,16 +4135,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="28.8" customWidth="1" min="4" max="4"/>
+    <col width="29.7" customWidth="1" min="4" max="4"/>
     <col width="58.5" customWidth="1" min="5" max="5"/>
     <col width="9.9" customWidth="1" min="6" max="6"/>
-    <col width="15.3" customWidth="1" min="7" max="7"/>
+    <col width="27.9" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -4469,8 +4526,218 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>D-09</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Ngưỡng món trễ: Bếp nóng 15' · Bếp lạnh 10' · Quầy nước 5'; đỏ ở 1,5 × ngưỡng</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Một ngưỡng chung 15'</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Món lạnh, đồ uống phải ra nhanh hơn món nóng</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>MOM-02 (Elicitation Results §5)</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>BR-06, KDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>D-10</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Đơn mang về thanh toán đủ trước khi gửi bếp</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Trả khi nhận món</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Tránh khách bỏ đơn; thói quen hiện tại của quầy</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>CSH, MGR</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>MOM-02</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>BR-13, UC-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>D-11</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>24/11/2026</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Thêm tìm kiếm không dấu, nút Hoàn tác cho Bếp trưởng, cảnh báo món chứa chất dị ứng trên app phục vụ</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Giữ thiết kế ban đầu</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>3 lỗi mức Cao trong user testing</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>PO</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>UX Evaluation §3</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>UC-01, UC-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>D-12</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>24/11/2026</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>KDS nền tối, chữ ≥ 20 px, mỗi món là một vùng chạm lớn</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Giao diện sáng như app phục vụ</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Bếp nóng, ẩm, tay ướt; đọc từ 1,5 m</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>CHF, BA</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>UX Evaluation §1</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>NFR-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>D-13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>26/02/2027</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Go-live 01/03/2027, chạy song song phiếu giấy 1 tuần làm dự phòng</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Lùi go-live; chuyển đổi từng phần</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>UAT đạt 100%, 0 lỗi mở</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>OWN</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>UAT Report §4</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Go-live Plan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H9"/>
+  <autoFilter ref="A1:H14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>